<commit_message>
260313D: Replace Stevens power law with exponential saturation model, Gauss-Newton fit, R2 metric, restore luxMax high-water mark
</commit_message>
<xml_diff>
--- a/excel/luxdata 1a..xlsx
+++ b/excel/luxdata 1a..xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Documents\PlatformIO\ESP32\Projects\Kwal27\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BFDBC4F-147F-4E80-8A6A-47A33D0C4D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2A36FC13-3C6E-461A-B95A-7620C782FB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17505" yWindow="8910" windowWidth="23370" windowHeight="21435" xr2:uid="{7CDCDC7A-177B-40E3-8BAD-B0D32D1552ED}"/>
   </bookViews>
@@ -593,11 +593,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -673,7 +674,17 @@
   <c:chart>
     <c:autoTitleDeleted val="1"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.1214838145231846"/>
+          <c:y val="5.8309037900874633E-2"/>
+          <c:w val="0.79715507436570432"/>
+          <c:h val="0.78463243115018788"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -1204,7 +1215,551 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>luxdata_130113!$P$2:$P$28</c:f>
+              <c:numCache>
+                <c:formatCode>_-* #,##0.0_-;\-* #,##0.0_-;_-* "-"??_-;_-@_-</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18.8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>36.700000000000003</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>60.7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>90.7</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>126.7</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>147</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>168.8</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>192</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>216.8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>243</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>270.8</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>319.8</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>200.4</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>102.8</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>15.7</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>10.6</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>43.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>luxdata_130113!$Q$2:$Q$28</c:f>
+              <c:numCache>
+                <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>5.9285725605226771</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>21.517203682192953</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46.134407203176828</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>75.58091848224224</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>107.76780220521955</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>138.78548344426471</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>166.86540525138531</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>190.76806032946956</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>209.5340484577938</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>223.65019385953391</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>233.54777185040564</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>240.20902622525321</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>244.41289693350805</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>246.96120541752126</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>248.41994300707117</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>249.21222210038891</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>249.62564063807534</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>249.82941798681091</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>249.92591476928533</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>249.96914754897833</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>249.98296591738276</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>249.38770377276026</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>238.55605329831025</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>124.60598273348612</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>93.905605397147184</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>68.099302896351134</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>181.7988847154059</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FA12-4D59-BA05-886746CA0A25}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>luxdata_130113!$M$22:$M$28</c:f>
+              <c:numCache>
+                <c:formatCode>_-* #,##0.0_-;\-* #,##0.0_-;_-* "-"??_-;_-@_-</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>319.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>200.4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>102.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15.7</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10.6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>43.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>luxdata_130113!$N$22:$N$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>256.47669999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>235.07309999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>207.92460000000003</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>90.772499999999994</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>68.394300000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>88.030799999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>216.01160000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-FA12-4D59-BA05-886746CA0A25}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1892519759"/>
+        <c:axId val="1892520239"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1892519759"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="LID4096"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1892520239"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1892520239"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="LID4096"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1892519759"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="LID4096"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1760,20 +2315,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>314325</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1793,6 +2864,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>323850</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{560BA08A-E3D7-D2D4-024D-8322D64C30C8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2098,13 +3205,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABE533AC-5832-406A-966C-5F2B9F8D5059}">
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="4" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2136,8 +3243,14 @@
         <f>D1&amp;"*"&amp;E1</f>
         <v>brightness*nf</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="Q1">
+        <v>250</v>
+      </c>
+      <c r="R1">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2169,8 +3282,16 @@
         <f>D2*E2</f>
         <v>237.3</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P2" s="3">
+        <f>M2</f>
+        <v>0.8</v>
+      </c>
+      <c r="Q2" s="4">
+        <f>$Q$1*(1-EXP(-$R$1*M2))</f>
+        <v>5.9285725605226771</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2202,8 +3323,16 @@
         <f t="shared" ref="N3:N29" si="6">D3*E3</f>
         <v>256.60000000000002</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P3" s="3">
+        <f t="shared" ref="P3:P28" si="7">M3</f>
+        <v>3</v>
+      </c>
+      <c r="Q3" s="4">
+        <f t="shared" ref="Q3:Q37" si="8">$Q$1*(1-EXP(-$R$1*M3))</f>
+        <v>21.517203682192953</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2235,8 +3364,16 @@
         <f t="shared" si="6"/>
         <v>270.7</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P4" s="3">
+        <f t="shared" si="7"/>
+        <v>6.8</v>
+      </c>
+      <c r="Q4" s="4">
+        <f t="shared" si="8"/>
+        <v>46.134407203176828</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2268,8 +3405,16 @@
         <f t="shared" si="6"/>
         <v>282.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P5" s="3">
+        <f t="shared" si="7"/>
+        <v>12</v>
+      </c>
+      <c r="Q5" s="4">
+        <f t="shared" si="8"/>
+        <v>75.58091848224224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2301,8 +3446,16 @@
         <f t="shared" si="6"/>
         <v>292</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P6" s="3">
+        <f t="shared" si="7"/>
+        <v>18.8</v>
+      </c>
+      <c r="Q6" s="4">
+        <f t="shared" si="8"/>
+        <v>107.76780220521955</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -2334,8 +3487,16 @@
         <f t="shared" si="6"/>
         <v>300.8</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P7" s="3">
+        <f t="shared" si="7"/>
+        <v>27</v>
+      </c>
+      <c r="Q7" s="4">
+        <f t="shared" si="8"/>
+        <v>138.78548344426471</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -2367,8 +3528,16 @@
         <f t="shared" si="6"/>
         <v>308.60000000000002</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P8" s="3">
+        <f t="shared" si="7"/>
+        <v>36.700000000000003</v>
+      </c>
+      <c r="Q8" s="4">
+        <f t="shared" si="8"/>
+        <v>166.86540525138531</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2400,8 +3569,16 @@
         <f t="shared" si="6"/>
         <v>315.89999999999998</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P9" s="3">
+        <f t="shared" si="7"/>
+        <v>48</v>
+      </c>
+      <c r="Q9" s="4">
+        <f t="shared" si="8"/>
+        <v>190.76806032946956</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2433,8 +3610,16 @@
         <f t="shared" si="6"/>
         <v>322.60000000000002</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P10" s="3">
+        <f t="shared" si="7"/>
+        <v>60.7</v>
+      </c>
+      <c r="Q10" s="4">
+        <f t="shared" si="8"/>
+        <v>209.5340484577938</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -2466,8 +3651,16 @@
         <f t="shared" si="6"/>
         <v>328.9</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P11" s="3">
+        <f t="shared" si="7"/>
+        <v>75</v>
+      </c>
+      <c r="Q11" s="4">
+        <f t="shared" si="8"/>
+        <v>223.65019385953391</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2499,8 +3692,16 @@
         <f t="shared" si="6"/>
         <v>334.8</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P12" s="3">
+        <f t="shared" si="7"/>
+        <v>90.7</v>
+      </c>
+      <c r="Q12" s="4">
+        <f t="shared" si="8"/>
+        <v>233.54777185040564</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2532,8 +3733,16 @@
         <f t="shared" si="6"/>
         <v>340.4</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P13" s="3">
+        <f t="shared" si="7"/>
+        <v>108</v>
+      </c>
+      <c r="Q13" s="4">
+        <f t="shared" si="8"/>
+        <v>240.20902622525321</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -2565,8 +3774,16 @@
         <f t="shared" si="6"/>
         <v>345.7</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P14" s="3">
+        <f t="shared" si="7"/>
+        <v>126.7</v>
+      </c>
+      <c r="Q14" s="4">
+        <f t="shared" si="8"/>
+        <v>244.41289693350805</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -2598,8 +3815,16 @@
         <f t="shared" si="6"/>
         <v>350.8</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P15" s="3">
+        <f t="shared" si="7"/>
+        <v>147</v>
+      </c>
+      <c r="Q15" s="4">
+        <f t="shared" si="8"/>
+        <v>246.96120541752126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -2631,8 +3856,16 @@
         <f t="shared" si="6"/>
         <v>355.7</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P16" s="3">
+        <f t="shared" si="7"/>
+        <v>168.8</v>
+      </c>
+      <c r="Q16" s="4">
+        <f t="shared" si="8"/>
+        <v>248.41994300707117</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -2664,8 +3897,16 @@
         <f t="shared" si="6"/>
         <v>360.4</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P17" s="3">
+        <f t="shared" si="7"/>
+        <v>192</v>
+      </c>
+      <c r="Q17" s="4">
+        <f t="shared" si="8"/>
+        <v>249.21222210038891</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2697,8 +3938,16 @@
         <f t="shared" si="6"/>
         <v>364.9</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P18" s="3">
+        <f t="shared" si="7"/>
+        <v>216.8</v>
+      </c>
+      <c r="Q18" s="4">
+        <f t="shared" si="8"/>
+        <v>249.62564063807534</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2730,8 +3979,16 @@
         <f t="shared" si="6"/>
         <v>369.2</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P19" s="3">
+        <f t="shared" si="7"/>
+        <v>243</v>
+      </c>
+      <c r="Q19" s="4">
+        <f t="shared" si="8"/>
+        <v>249.82941798681091</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2763,8 +4020,16 @@
         <f t="shared" si="6"/>
         <v>373.4</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P20" s="3">
+        <f t="shared" si="7"/>
+        <v>270.8</v>
+      </c>
+      <c r="Q20" s="4">
+        <f t="shared" si="8"/>
+        <v>249.92591476928533</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2796,8 +4061,16 @@
         <f t="shared" si="6"/>
         <v>377.5</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P21" s="3">
+        <f t="shared" si="7"/>
+        <v>300</v>
+      </c>
+      <c r="Q21" s="4">
+        <f t="shared" si="8"/>
+        <v>249.96914754897833</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2829,8 +4102,16 @@
         <f t="shared" si="6"/>
         <v>256.47669999999999</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P22" s="3">
+        <f t="shared" si="7"/>
+        <v>319.8</v>
+      </c>
+      <c r="Q22" s="4">
+        <f t="shared" si="8"/>
+        <v>249.98296591738276</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -2862,8 +4143,16 @@
         <f t="shared" si="6"/>
         <v>235.07309999999998</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P23" s="3">
+        <f t="shared" si="7"/>
+        <v>200.4</v>
+      </c>
+      <c r="Q23" s="4">
+        <f t="shared" si="8"/>
+        <v>249.38770377276026</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -2895,8 +4184,16 @@
         <f t="shared" si="6"/>
         <v>207.92460000000003</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P24" s="3">
+        <f t="shared" si="7"/>
+        <v>102.8</v>
+      </c>
+      <c r="Q24" s="4">
+        <f t="shared" si="8"/>
+        <v>238.55605329831025</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -2928,8 +4225,16 @@
         <f t="shared" si="6"/>
         <v>90.772499999999994</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P25" s="3">
+        <f t="shared" si="7"/>
+        <v>23</v>
+      </c>
+      <c r="Q25" s="4">
+        <f t="shared" si="8"/>
+        <v>124.60598273348612</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -2961,8 +4266,16 @@
         <f t="shared" si="6"/>
         <v>68.394300000000001</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P26" s="3">
+        <f t="shared" si="7"/>
+        <v>15.7</v>
+      </c>
+      <c r="Q26" s="4">
+        <f t="shared" si="8"/>
+        <v>93.905605397147184</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -2994,8 +4307,16 @@
         <f t="shared" si="6"/>
         <v>88.030799999999999</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P27" s="3">
+        <f t="shared" si="7"/>
+        <v>10.6</v>
+      </c>
+      <c r="Q27" s="4">
+        <f t="shared" si="8"/>
+        <v>68.099302896351134</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -3027,8 +4348,16 @@
         <f t="shared" si="6"/>
         <v>216.01160000000002</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P28" s="3">
+        <f t="shared" si="7"/>
+        <v>43.3</v>
+      </c>
+      <c r="Q28" s="4">
+        <f t="shared" si="8"/>
+        <v>181.7988847154059</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C29" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3049,16 +4378,13 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M29" s="3" t="e">
-        <f t="shared" si="5"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N29" t="e">
-        <f t="shared" si="6"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M29" s="3"/>
+      <c r="Q29" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C30" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3079,8 +4405,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="Q30" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C31" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3101,8 +4431,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="Q31" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C32" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3123,8 +4457,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="33" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="Q32" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C33" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3145,8 +4483,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="34" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="Q33" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C34" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3167,8 +4509,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="35" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="Q34" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C35" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3189,8 +4535,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="36" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="Q35" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C36" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3211,8 +4561,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="37" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="Q36" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C37" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3233,8 +4587,12 @@
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="38" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="Q37" s="4">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C38" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3256,7 +4614,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="39" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C39" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3278,7 +4636,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="40" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C40" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3300,7 +4658,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="41" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C41" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3322,7 +4680,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="42" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C42" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3344,7 +4702,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="43" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C43" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3366,7 +4724,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="44" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C44" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3388,7 +4746,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="45" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C45" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3410,7 +4768,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="46" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C46" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3432,7 +4790,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="47" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C47" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
@@ -3454,7 +4812,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="48" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C48" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>

</xml_diff>